<commit_message>
Add weekly cumulative summary table to reports and tally
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 20:08:08</t>
+          <t>2026-05-14 20:34:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,24 +482,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.14</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+          <t>4.07</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Strava</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>View</t>
@@ -507,14 +499,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Manual Fix</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14 20:34:20</t>
+          <t>2026-05-17 12:33:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -524,34 +516,36 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.07</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+          <t>5.91</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
         <is>
           <t>View</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Manual Fix</t>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-17 12:33:11</t>
+          <t>2026-05-18 20:08:08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -561,12 +555,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.91</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -576,10 +570,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>View</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -628,7 +632,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.14</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -660,7 +664,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>5.91</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -698,7 +702,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.14</v>
+        <v>14.12</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: remove exposed API key, verify Kelvin entry, reset Week 21 points (scoring starts Week 22)
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -708,7 +708,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Week 22/23: Add Surya (51,942 steps), Chee (69,621 steps), Kelvin 10.44km, Jeremy 10.97km+7.23km, CRX 3.52km run; add Tesseract OCR fallback
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14 20:34:20</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,21 +571,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.07</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>44,238</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>fitness app</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>View</t>
@@ -593,14 +601,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Manual Fix</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-17 12:33:11</t>
+          <t>2026-06-02 20:32:59</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -610,21 +618,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.91</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>3.52</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>View</t>
@@ -679,7 +695,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8.210000000000001</v>
+        <v>7.66</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -711,10 +727,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.91</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>29156</v>
+        <v>73394</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -749,10 +765,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.12</v>
+        <v>7.66</v>
       </c>
       <c r="C6" t="n">
-        <v>29156</v>
+        <v>73394</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: correct app to Strava for Chun Chieh, Jeremy (6/4, 6/5) - all verified
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25 16:56:39</t>
+          <t>2026-05-18 20:08:08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,17 +477,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29,156</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01 09:09:44</t>
+          <t>2026-05-25 16:56:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44,238</t>
+          <t>29,156</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>fitness app</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 20:08:08</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>44,238</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>fitness app</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
fix: CRX pledge=Steps (not Distance), Jeremy 6/6 distance=7.46km, Kelvin 6/7 Strava verified, fix pledge detection across months
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25 16:56:39</t>
+          <t>2026-05-18 20:08:08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,17 +477,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29,156</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01 09:09:44</t>
+          <t>2026-05-25 16:56:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44,238</t>
+          <t>29,156</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>fitness app</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 20:08:08</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>44,238</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>fitness app</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
fix: CRX total steps=47,250 (includes 3,012 from run entry), Tier 1 = 1pt
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3,012</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -698,7 +698,7 @@
         <v>7.66</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>3012</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -768,7 +768,7 @@
         <v>7.66</v>
       </c>
       <c r="C6" t="n">
-        <v>73394</v>
+        <v>76406</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: CRX 4 new activities (20,024 steps) - June total 67,274 steps = Tier 3 (3pts)
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,6 +647,194 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>6/7/2026 19:14:51</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5.51</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4,532</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6/7/2026 19:14:51</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4.42</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5,470</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6/7/2026 19:14:51</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4.01</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3,398</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6/7/2026 19:14:51</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4.75</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>6,624</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -695,10 +883,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.66</v>
+        <v>26.35</v>
       </c>
       <c r="C2" t="n">
-        <v>3012</v>
+        <v>23036</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -765,10 +953,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.66</v>
+        <v>26.35</v>
       </c>
       <c r="C6" t="n">
-        <v>76406</v>
+        <v>96430</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: CRX Healthy 365 weekly steps 99,091 (week of 1 Jun) = Tier 5 = 5pts, total 26
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,7 +608,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-02 20:32:59</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -618,17 +618,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.52</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3,012</t>
+          <t>44,238</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -655,7 +655,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6/7/2026 19:14:51</t>
+          <t>2026-06-02 20:32:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>3.52</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4,532</t>
+          <t>3,012</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.42</t>
+          <t>5.51</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5,470</t>
+          <t>4,532</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -764,12 +764,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.01</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3,398</t>
+          <t>5,470</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -811,30 +811,124 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>4.01</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>3,398</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6/7/2026 19:14:51</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>4.75</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>6,624</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Strava</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>View</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6/8/2026 06:03:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CRX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>99,091</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Healthy 365</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -918,7 +1012,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>73394</v>
+        <v>216723</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -956,7 +1050,7 @@
         <v>26.35</v>
       </c>
       <c r="C6" t="n">
-        <v>96430</v>
+        <v>239759</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: weekly cumulative scoring resets each week, no carryover between weeks
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25 16:56:39</t>
+          <t>2026-05-18 20:08:08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,17 +477,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29,156</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01 09:09:44</t>
+          <t>2026-05-25 16:56:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44,238</t>
+          <t>29,156</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>fitness app</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 20:08:08</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,17 +571,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>44,238</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>fitness app</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -608,7 +608,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-01 09:09:44</t>
+          <t>2026-06-02 20:32:59</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -618,17 +618,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>3.52</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>44,238</t>
+          <t>3,012</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -655,7 +655,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-02 20:32:59</t>
+          <t>6/7/2026 19:14:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.52</t>
+          <t>5.51</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3,012</t>
+          <t>4,532</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4,532</t>
+          <t>5,470</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -764,12 +764,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.42</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5,470</t>
+          <t>3,398</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4.01</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3,398</t>
+          <t>6,624</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6/7/2026 19:14:51</t>
+          <t>6/8/2026 06:03:23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -853,17 +853,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>6,624</t>
+          <t>99,091</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -890,7 +890,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6/8/2026 06:03:23</t>
+          <t>6/8/2026 6:03:23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>99,091</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -930,14 +930,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Committee Approval Required</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6/8/2026 6:03:23</t>
+          <t>6/8/2026 9:39:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -976,53 +976,6 @@
         </is>
       </c>
       <c r="I12" t="inlineStr">
-        <is>
-          <t>Committee Approval Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>6/8/2026 9:39:05</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CRX</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
         <is>
           <t>Committee Approval Required</t>
         </is>
@@ -1106,7 +1059,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>216723</v>
+        <v>172485</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1144,7 +1097,7 @@
         <v>26.35</v>
       </c>
       <c r="C6" t="n">
-        <v>239759</v>
+        <v>195521</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: Week 24 shows only this week's entries and scores, no carryover
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -884,100 +884,6 @@
       <c r="I10" t="inlineStr">
         <is>
           <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>6/8/2026 6:03:23</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CRX</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Committee Approval Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>6/8/2026 9:39:05</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CRX</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Committee Approval Required</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: Week 24 - Jeremy 7.44km (6/12)
</commit_message>
<xml_diff>
--- a/Reports/Members/CRX_Activity_Report.xlsx
+++ b/Reports/Members/CRX_Activity_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25 16:56:39</t>
+          <t>2026-05-18 20:08:08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,17 +477,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Run/Jog</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29,156</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Healthy 365</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01 09:09:44</t>
+          <t>2026-05-25 16:56:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44,238</t>
+          <t>29,156</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>fitness app</t>
+          <t>Healthy 365</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 20:08:08</t>
+          <t>2026-06-01 09:09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Run/Jog</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>44,238</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>fitness app</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>